<commit_message>
Catch right censored observations with a found or not found variable.
</commit_message>
<xml_diff>
--- a/goanna_burrow_detection.xlsx
+++ b/goanna_burrow_detection.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -689,7 +689,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Time taken to find the burrow</t>
+          <t>Time spent searching for a burrow, whether or not one was found</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -728,12 +728,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>dig_or_inspect</t>
+          <t>burrow_found</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Was the burrow dug or just inspected?</t>
+          <t>Was a burrow found?</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -745,52 +745,79 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>select_multiple found_choices</t>
+          <t>select_one dig_or_inspect_choices</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>what_did_you_find</t>
+          <t>dig_or_inspect</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>What did you find?</t>
+          <t>Was the burrow dug or just inspected?</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>${dig_or_inspect} = 'Yes'</t>
+          <t>${burrow_found} = 'Yes'</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>select_multiple found_choices</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>what_did_you_find</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>What did you find?</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>${burrow_found} = 'Yes' and ${dig_or_inspect} = 'Yes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>what_did_you_find_other</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Please specify</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>selected(${what_did_you_find}, 'other')</t>
         </is>

</xml_diff>

<commit_message>
Add burrow-type and notes fields to the record sheet
Field-team feedback (update-notes.txt items 8-9):

- Burrow type: when a burrow is found, record whether it's a Wandidji
  (V. acanthurus) or Wanggali (V. gouldii) burrow, or Other with a
  free-text box. Shown only when burrow_found = Yes, defaults to
  Wandidji (the overwhelmingly common type, so no "please select"
  validation), and resets to that default when burrow_found flips
  back to No.
- Notes: an always-visible free-text field for observations that
  don't fit a category.

XLSForm gains a burrow_type_choices list and a `default` column;
new survey rows burrow_type / burrow_type_other (relevant on
burrow_type = 'other') / notes, placed to match buildSubmissionXml
element order. Re-validated with xls2xform.

sw.js CACHE_NAME bumped v12 -> v13.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019EhNnzhxQDRbaie1534wzj
</commit_message>
<xml_diff>
--- a/goanna_burrow_detection.xlsx
+++ b/goanna_burrow_detection.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -479,6 +479,11 @@
           <t>relevant</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -767,17 +772,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>select_one yes_no_choices</t>
+          <t>select_one burrow_type_choices</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>dig_or_inspect</t>
+          <t>burrow_type</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Was the burrow inspected?</t>
+          <t>What type of burrow?</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -788,87 +793,168 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>${burrow_found} = 'Yes'</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>wandidji</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>select_one inspect_method_choices</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>inspection_method</t>
+          <t>burrow_type_other</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>How was the burrow inspected?</t>
+          <t>Please specify</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>${dig_or_inspect} = 'Yes'</t>
+          <t>${burrow_type} = 'other'</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>select_multiple found_choices</t>
+          <t>select_one yes_no_choices</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>what_did_you_find</t>
+          <t>dig_or_inspect</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>What did you find?</t>
+          <t>Was the burrow inspected?</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>${dig_or_inspect} = 'Yes'</t>
+          <t>${burrow_found} = 'Yes'</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>select_one inspect_method_choices</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>inspection_method</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>How was the burrow inspected?</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>${dig_or_inspect} = 'Yes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>select_multiple found_choices</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>what_did_you_find</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>What did you find?</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>${dig_or_inspect} = 'Yes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>what_did_you_find_other</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Please specify</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>selected(${what_did_you_find}, 'other')</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -883,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1089,6 +1175,57 @@
         </is>
       </c>
       <c r="C12" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>burrow_type_choices</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>wandidji</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Wandidji (V. acanthurus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>burrow_type_choices</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>wanggali</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Wanggali (V. gouldii)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>burrow_type_choices</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>Other</t>
         </is>

</xml_diff>